<commit_message>
feat: add Investors, Stocks, and SignalScore pages from Excel data
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/GoldSignal_Stocks.xlsx
+++ b/GoldSignal_Stocks.xlsx
@@ -1,140 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jonjo\gold-signal\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F917C64B-2ABA-452C-9184-414D4BA276BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
   <sheets>
     <sheet name="Stocks" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="36">
-  <si>
-    <t>Ticker</t>
-  </si>
-  <si>
-    <t>Company</t>
-  </si>
-  <si>
-    <t>Sector</t>
-  </si>
-  <si>
-    <t>Weekly Change (%)</t>
-  </si>
-  <si>
-    <t>Signal Score</t>
-  </si>
-  <si>
-    <t>NEM</t>
-  </si>
-  <si>
-    <t>Newmont Corporation</t>
-  </si>
-  <si>
-    <t>Gold Mining</t>
-  </si>
-  <si>
-    <t>FNV</t>
-  </si>
-  <si>
-    <t>Franco-Nevada Corp</t>
-  </si>
-  <si>
-    <t>Royalty &amp; Streaming</t>
-  </si>
-  <si>
-    <t>WPM</t>
-  </si>
-  <si>
-    <t>Wheaton Precious Metals</t>
-  </si>
-  <si>
-    <t>Silver Streaming</t>
-  </si>
-  <si>
-    <t>GOLD</t>
-  </si>
-  <si>
-    <t>Barrick Gold Corporation</t>
-  </si>
-  <si>
-    <t>AEM</t>
-  </si>
-  <si>
-    <t>Agnico Eagle Mines</t>
-  </si>
-  <si>
-    <t>KGC</t>
-  </si>
-  <si>
-    <t>Kinross Gold</t>
-  </si>
-  <si>
-    <t>AG</t>
-  </si>
-  <si>
-    <t>First Majestic Silver</t>
-  </si>
-  <si>
-    <t>Silver Mining</t>
-  </si>
-  <si>
-    <t>PAAS</t>
-  </si>
-  <si>
-    <t>Pan American Silver</t>
-  </si>
-  <si>
-    <t>RGLD</t>
-  </si>
-  <si>
-    <t>Royal Gold</t>
-  </si>
-  <si>
-    <t>GDX</t>
-  </si>
-  <si>
-    <t>VanEck Gold Miners ETF</t>
-  </si>
-  <si>
-    <t>ETF</t>
-  </si>
-  <si>
-    <t>HL</t>
-  </si>
-  <si>
-    <t>Hecla Mining</t>
-  </si>
-  <si>
-    <t>MUX</t>
-  </si>
-  <si>
-    <t>McEwen Mining</t>
-  </si>
-  <si>
-    <t>ELE</t>
-  </si>
-  <si>
-    <t>Elemental Royalty</t>
-  </si>
-</sst>
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <numFmts count="1">
+    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+  </numFmts>
+  <fonts count="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -164,21 +65,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -503,43 +396,42 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.796875" customWidth="1"/>
-    <col min="2" max="2" width="32.796875" customWidth="1"/>
-    <col min="3" max="3" width="22.796875" customWidth="1"/>
-    <col min="4" max="4" width="18.796875" customWidth="1"/>
-    <col min="5" max="5" width="14.796875" customWidth="1"/>
+    <col min="1" max="1" width="8.83203125" customWidth="1"/>
+    <col min="2" max="2" width="32.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C2" t="s">
-        <v>10</v>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Ticker</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Company</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Sector</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Monthly Change (%)</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Signal Score</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>ELE</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Elemental Royalty</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Royalty &amp; Streaming</v>
       </c>
       <c r="D2">
         <v>23</v>
@@ -548,15 +440,15 @@
         <v>99</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" t="s">
-        <v>10</v>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>FNV</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Franco-Nevada Corp</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Royalty &amp; Streaming</v>
       </c>
       <c r="D3">
         <v>1.8</v>
@@ -565,15 +457,15 @@
         <v>91</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" t="s">
-        <v>13</v>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>WPM</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Wheaton Precious Metals</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Silver Streaming</v>
       </c>
       <c r="D4">
         <v>3.1</v>
@@ -582,15 +474,15 @@
         <v>89</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>7</v>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>GOLD</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Barrick Gold Corporation</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Gold Mining</v>
       </c>
       <c r="D5">
         <v>-0.6</v>
@@ -599,15 +491,15 @@
         <v>87</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" t="s">
-        <v>7</v>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>AEM</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Agnico Eagle Mines</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Gold Mining</v>
       </c>
       <c r="D6">
         <v>1.2</v>
@@ -616,15 +508,15 @@
         <v>85</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" t="s">
-        <v>7</v>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>KGC</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Kinross Gold</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Gold Mining</v>
       </c>
       <c r="D7">
         <v>0.9</v>
@@ -633,15 +525,15 @@
         <v>83</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" t="s">
-        <v>22</v>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>AG</v>
+      </c>
+      <c r="B8" t="str">
+        <v>First Majestic Silver</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Silver Mining</v>
       </c>
       <c r="D8">
         <v>4.2</v>
@@ -650,32 +542,32 @@
         <v>81</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B9" t="s">
-        <v>24</v>
-      </c>
-      <c r="C9" t="s">
-        <v>22</v>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>PAAS</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Pan American Silver</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Silver Mining</v>
       </c>
       <c r="D9">
-        <v>-1.1000000000000001</v>
+        <v>-1.1</v>
       </c>
       <c r="E9">
         <v>78</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>25</v>
-      </c>
-      <c r="B10" t="s">
-        <v>26</v>
-      </c>
-      <c r="C10" t="s">
-        <v>10</v>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>RGLD</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Royal Gold</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Royalty &amp; Streaming</v>
       </c>
       <c r="D10">
         <v>0</v>
@@ -684,15 +576,15 @@
         <v>76</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B11" t="s">
-        <v>28</v>
-      </c>
-      <c r="C11" t="s">
-        <v>29</v>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>GDX</v>
+      </c>
+      <c r="B11" t="str">
+        <v>VanEck Gold Miners ETF</v>
+      </c>
+      <c r="C11" t="str">
+        <v>ETF</v>
       </c>
       <c r="D11">
         <v>2</v>
@@ -701,32 +593,32 @@
         <v>72</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B12" t="s">
-        <v>31</v>
-      </c>
-      <c r="C12" t="s">
-        <v>22</v>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>HL</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Hecla Mining</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Silver Mining</v>
       </c>
       <c r="D12">
-        <v>-2.2999999999999998</v>
+        <v>-2.3</v>
       </c>
       <c r="E12">
         <v>58</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>32</v>
-      </c>
-      <c r="B13" t="s">
-        <v>33</v>
-      </c>
-      <c r="C13" t="s">
-        <v>7</v>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>MUX</v>
+      </c>
+      <c r="B13" t="str">
+        <v>McEwen Mining</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Gold Mining</v>
       </c>
       <c r="D13">
         <v>-3.5</v>
@@ -735,15 +627,15 @@
         <v>52</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>5</v>
-      </c>
-      <c r="B14" t="s">
-        <v>6</v>
-      </c>
-      <c r="C14" t="s">
-        <v>7</v>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>NEM</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Newmont Corporation</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Gold Mining</v>
       </c>
       <c r="D14">
         <v>-22</v>
@@ -753,9 +645,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:C1 A3:E13 E1" numberStoredAsText="1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>